<commit_message>
Added new modified ropke and cordeau instances, and new Sun (selective PDP) instances (with code to read them). Also added outputting of statistics.
</commit_message>
<xml_diff>
--- a/Branch and Price/bnp_pricing_comparison_cgall_mip_nomip.xlsx
+++ b/Branch and Price/bnp_pricing_comparison_cgall_mip_nomip.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baubaid/Code_Work/PDP_Offline_Scheduling/Branch and Price/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5506129-2CF6-D44A-BD31-6B2D0E41D3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECBE5B98-E73A-2343-8519-FAF9DBEC75B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="46080" windowHeight="25320" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1280" yWindow="1320" windowWidth="38400" windowHeight="21000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BnP_GS_mip" sheetId="1" r:id="rId1"/>

</xml_diff>